<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-3-25.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-3-25.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-3-25.xlsx
@@ -1483,6 +1483,9 @@
       <c r="C121" t="str">
         <v>439_九星叶_undefined_undefined_1bunch</v>
       </c>
+      <c r="F121" t="str">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -1541,7 +1544,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0345102817101712155555347902010541220985846102351071012125481011112771012197510123221211586412282534265551881556182911161210205355855202084125713151530914610128920515101015151010155100</v>
+        <v>0345102817101712155555347902010541220985846102351071012125481011112771012197510123221211586412282534265551881556182911161210205355855202084125713151530914610128920515101015151010155102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>